<commit_message>
test algoritmi non vincolati iniziali
</commit_message>
<xml_diff>
--- a/exploratory_data_analisys/dimensions_reduction/risultati/correlazioni_dispersioni/matrice_correlazione.xlsx
+++ b/exploratory_data_analisys/dimensions_reduction/risultati/correlazioni_dispersioni/matrice_correlazione.xlsx
@@ -425,76 +425,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>IslandArea</t>
+          <t>Densità_pop</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Densità_pop</t>
+          <t>evi</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>evi</t>
+          <t>eolico</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>eolico</t>
+          <t>eolico_std</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>eolico_std</t>
+          <t>offshore</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>offshore</t>
+          <t>gdp_pro_capite</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>gdp_pro_capite</t>
+          <t>geothermal_potential</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>geothermal_potential</t>
+          <t>hydro</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>hydro</t>
+          <t>temp</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>temp</t>
+          <t>solar_pow</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>solar_pow</t>
+          <t>solar_seas_ind</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>solar_seas_ind</t>
+          <t>superficie_res</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>superficie_res</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>gdp_pop_urban_merged</t>
         </is>
@@ -503,686 +498,598 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>IslandArea</t>
+          <t>Densità_pop</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.04493181898450962</v>
+        <v>-0.1456033772007568</v>
       </c>
       <c r="D2" t="n">
-        <v>0.06269640499425402</v>
+        <v>-0.0386444791826261</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.05716260179848934</v>
+        <v>-0.002882600313852715</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.03423136919851529</v>
+        <v>-0.04035047138908179</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5330536100799442</v>
+        <v>0.0103976195557689</v>
       </c>
       <c r="H2" t="n">
-        <v>0.05552533860160565</v>
+        <v>-0.01270287605049416</v>
       </c>
       <c r="I2" t="n">
-        <v>0.04203575712036502</v>
+        <v>-0.02018417697929265</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5718754782474768</v>
+        <v>0.0655937961450038</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.08777209459367555</v>
+        <v>0.05391174584077664</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.06048329863432983</v>
+        <v>-0.05600307509311708</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.004563937708362182</v>
+        <v>-0.03091860644949788</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.06365188075385719</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.4392329713618456</v>
+        <v>0.1940996913778291</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Densità_pop</t>
+          <t>evi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.04493181898450962</v>
+        <v>-0.1456033772007568</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.1456033772007568</v>
+        <v>-0.07804394797776851</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0386444791826261</v>
+        <v>0.1102022605438197</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.002882600313852715</v>
+        <v>-0.1041258286466655</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.04035047138908179</v>
+        <v>-0.3768984365207781</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0103976195557689</v>
+        <v>-0.03986707901417107</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.01270287605049416</v>
+        <v>0.01634077623741607</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.02018417697929265</v>
+        <v>0.3540270520001535</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0655937961450038</v>
+        <v>-0.01352937325599825</v>
       </c>
       <c r="L3" t="n">
-        <v>0.05391174584077664</v>
+        <v>-0.1605073527495656</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.05600307509311708</v>
+        <v>0.009271703917644493</v>
       </c>
       <c r="N3" t="n">
-        <v>0.05034897530674703</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.1940996913778291</v>
+        <v>0.0604906980583572</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>evi</t>
+          <t>eolico</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.06269640499425402</v>
+        <v>-0.0386444791826261</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.1456033772007568</v>
+        <v>-0.07804394797776851</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.07804394797776851</v>
+        <v>-0.3904905114205633</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1102022605438197</v>
+        <v>0.2564129871631383</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.1041258286466655</v>
+        <v>0.3333822472966903</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.3768984365207781</v>
+        <v>-0.006835690923019978</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.03986707901417107</v>
+        <v>-0.04430470311093584</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01634077623741607</v>
+        <v>-0.3479335926520875</v>
       </c>
       <c r="K4" t="n">
-        <v>0.3540270520001535</v>
+        <v>-0.1972055437614216</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.01352937325599825</v>
+        <v>0.2178107841466263</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.1605073527495656</v>
+        <v>-0.002847214807961977</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.2163144824324924</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.0604906980583572</v>
+        <v>-0.03071466180415533</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>eolico</t>
+          <t>eolico_std</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.05716260179848934</v>
+        <v>-0.002882600313852715</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.0386444791826261</v>
+        <v>0.1102022605438197</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.07804394797776851</v>
+        <v>-0.3904905114205633</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.3904905114205633</v>
+        <v>-0.236939642745481</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2564129871631383</v>
+        <v>-0.3740466364527545</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3333822472966903</v>
+        <v>0.02023879606983839</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.006835690923019978</v>
+        <v>0.003329540816539707</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.04430470311093584</v>
+        <v>0.4057565423170194</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.3479335926520875</v>
+        <v>0.1299171412307018</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.1972055437614216</v>
+        <v>-0.1044963156843923</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2178107841466263</v>
+        <v>-0.05859774974580727</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1321416088647652</v>
-      </c>
-      <c r="O5" t="n">
-        <v>-0.03071466180415534</v>
+        <v>-0.04134193923629654</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>eolico_std</t>
+          <t>offshore</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.03423136919851529</v>
+        <v>-0.04035047138908179</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.002882600313852715</v>
+        <v>-0.1041258286466655</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1102022605438197</v>
+        <v>0.2564129871631383</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.3904905114205633</v>
+        <v>-0.236939642745481</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.236939642745481</v>
+        <v>0.3015311196530265</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.3740466364527545</v>
+        <v>0.02787838947075083</v>
       </c>
       <c r="I6" t="n">
-        <v>0.02023879606983839</v>
+        <v>0.1479122709797734</v>
       </c>
       <c r="J6" t="n">
-        <v>0.003329540816539707</v>
+        <v>-0.3944119310105226</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4057565423170194</v>
+        <v>-0.2013418226373828</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1299171412307018</v>
+        <v>0.1212480898397185</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.1044963156843923</v>
+        <v>0.5561087836388242</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.08563968501436756</v>
-      </c>
-      <c r="O6" t="n">
-        <v>-0.04134193923629658</v>
+        <v>0.1959009620477364</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>offshore</t>
+          <t>gdp_pro_capite</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5330536100799442</v>
+        <v>0.0103976195557689</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.04035047138908179</v>
+        <v>-0.3768984365207781</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.1041258286466655</v>
+        <v>0.3333822472966903</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2564129871631383</v>
+        <v>-0.3740466364527545</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.236939642745481</v>
+        <v>0.3015311196530265</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3015311196530265</v>
+        <v>0.02054100481888916</v>
       </c>
       <c r="I7" t="n">
-        <v>0.02787838947075083</v>
+        <v>0.006614441028997577</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1479122709797734</v>
+        <v>-0.6970097388231949</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.3944119310105226</v>
+        <v>-0.4202658561250584</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.2013418226373828</v>
+        <v>0.3147057019203685</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1212480898397185</v>
+        <v>0.06381074297636763</v>
       </c>
       <c r="N7" t="n">
-        <v>0.01917596765100124</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.1959009620477364</v>
+        <v>0.05515280701772647</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>gdp_pro_capite</t>
+          <t>geothermal_potential</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.05552533860160565</v>
+        <v>-0.01270287605049416</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0103976195557689</v>
+        <v>-0.03986707901417107</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.3768984365207781</v>
+        <v>-0.006835690923019978</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3333822472966903</v>
+        <v>0.02023879606983839</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.3740466364527545</v>
+        <v>0.02787838947075083</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3015311196530265</v>
+        <v>0.02054100481888916</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.02054100481888916</v>
+        <v>0.02500066842630837</v>
       </c>
       <c r="J8" t="n">
-        <v>0.006614441028997577</v>
+        <v>-0.01543672175437564</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.6970097388231949</v>
+        <v>0.04004131284992362</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.4202658561250584</v>
+        <v>-0.007095745571080414</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3147057019203685</v>
+        <v>0.01722600742217536</v>
       </c>
       <c r="N8" t="n">
-        <v>0.03307085724047992</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.05515280701772651</v>
+        <v>0.02901894782023856</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>geothermal_potential</t>
+          <t>hydro</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.04203575712036502</v>
+        <v>-0.02018417697929265</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.01270287605049416</v>
+        <v>0.01634077623741607</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.03986707901417107</v>
+        <v>-0.04430470311093584</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.006835690923019978</v>
+        <v>0.003329540816539707</v>
       </c>
       <c r="F9" t="n">
-        <v>0.02023879606983839</v>
+        <v>0.1479122709797734</v>
       </c>
       <c r="G9" t="n">
-        <v>0.02787838947075083</v>
+        <v>0.006614441028997577</v>
       </c>
       <c r="H9" t="n">
-        <v>0.02054100481888916</v>
+        <v>0.02500066842630837</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0.02500066842630837</v>
+        <v>-0.03115892015530013</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.01543672175437564</v>
+        <v>-0.04566218407760123</v>
       </c>
       <c r="L9" t="n">
-        <v>0.04004131284992362</v>
+        <v>-0.0009689161339465025</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.007095745571080414</v>
+        <v>0.1185980394424829</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.0246404985988846</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.02901894782023856</v>
+        <v>0.2806493460516831</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>hydro</t>
+          <t>temp</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.5718754782474768</v>
+        <v>0.0655937961450038</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.02018417697929265</v>
+        <v>0.3540270520001535</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01634077623741607</v>
+        <v>-0.3479335926520875</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.04430470311093584</v>
+        <v>0.4057565423170194</v>
       </c>
       <c r="F10" t="n">
-        <v>0.003329540816539707</v>
+        <v>-0.3944119310105226</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1479122709797734</v>
+        <v>-0.6970097388231949</v>
       </c>
       <c r="H10" t="n">
-        <v>0.006614441028997577</v>
+        <v>-0.01543672175437564</v>
       </c>
       <c r="I10" t="n">
-        <v>0.02500066842630837</v>
+        <v>-0.03115892015530013</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.03115892015530013</v>
+        <v>0.6679941812612148</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.04566218407760123</v>
+        <v>-0.452280205443447</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.0009689161339465025</v>
+        <v>-0.08569332644826699</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.05268009763488148</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.2806493460516831</v>
+        <v>-0.008924192964144765</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>temp</t>
+          <t>solar_pow</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.08777209459367555</v>
+        <v>0.05391174584077664</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0655937961450038</v>
+        <v>-0.01352937325599825</v>
       </c>
       <c r="D11" t="n">
-        <v>0.3540270520001535</v>
+        <v>-0.1972055437614216</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.3479335926520875</v>
+        <v>0.1299171412307018</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4057565423170194</v>
+        <v>-0.2013418226373828</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.3944119310105226</v>
+        <v>-0.4202658561250584</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.6970097388231949</v>
+        <v>0.04004131284992362</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.01543672175437564</v>
+        <v>-0.04566218407760123</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.03115892015530013</v>
+        <v>0.6679941812612148</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6679941812612148</v>
+        <v>-0.4843575067089396</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.452280205443447</v>
+        <v>-0.02748265248561407</v>
       </c>
       <c r="N11" t="n">
-        <v>0.01960986702368907</v>
-      </c>
-      <c r="O11" t="n">
-        <v>-0.008924192964144761</v>
+        <v>0.01590378690918018</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>solar_pow</t>
+          <t>solar_seas_ind</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.06048329863432983</v>
+        <v>-0.05600307509311708</v>
       </c>
       <c r="C12" t="n">
-        <v>0.05391174584077664</v>
+        <v>-0.1605073527495656</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.01352937325599825</v>
+        <v>0.2178107841466263</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1972055437614216</v>
+        <v>-0.1044963156843923</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1299171412307018</v>
+        <v>0.1212480898397185</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.2013418226373828</v>
+        <v>0.3147057019203685</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.4202658561250584</v>
+        <v>-0.007095745571080414</v>
       </c>
       <c r="I12" t="n">
-        <v>0.04004131284992362</v>
+        <v>-0.0009689161339465025</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.04566218407760123</v>
+        <v>-0.452280205443447</v>
       </c>
       <c r="K12" t="n">
-        <v>0.6679941812612148</v>
+        <v>-0.4843575067089396</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.4843575067089396</v>
+        <v>0.003677052112265631</v>
       </c>
       <c r="N12" t="n">
-        <v>0.1265143597509155</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0.01590378690918017</v>
+        <v>-0.03043192147242368</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>solar_seas_ind</t>
+          <t>superficie_res</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.004563937708362182</v>
+        <v>-0.03091860644949788</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.05600307509311708</v>
+        <v>0.009271703917644493</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1605073527495656</v>
+        <v>-0.002847214807961977</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2178107841466263</v>
+        <v>-0.05859774974580727</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.1044963156843923</v>
+        <v>0.5561087836388242</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1212480898397185</v>
+        <v>0.06381074297636763</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3147057019203685</v>
+        <v>0.01722600742217536</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.007095745571080414</v>
+        <v>0.1185980394424829</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.0009689161339465025</v>
+        <v>-0.08569332644826699</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.452280205443447</v>
+        <v>-0.02748265248561407</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.4843575067089396</v>
+        <v>0.003677052112265631</v>
       </c>
       <c r="M13" t="n">
         <v>1</v>
       </c>
       <c r="N13" t="n">
-        <v>0.03535199604169725</v>
-      </c>
-      <c r="O13" t="n">
-        <v>-0.03043192147242368</v>
+        <v>0.2465594051809464</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>superficie_res</t>
+          <t>gdp_pop_urban_merged</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.06365188075385719</v>
+        <v>0.1940996913778291</v>
       </c>
       <c r="C14" t="n">
-        <v>0.05034897530674703</v>
+        <v>0.0604906980583572</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.2163144824324924</v>
+        <v>-0.03071466180415533</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1321416088647652</v>
+        <v>-0.04134193923629654</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.08563968501436756</v>
+        <v>0.1959009620477364</v>
       </c>
       <c r="G14" t="n">
-        <v>0.01917596765100124</v>
+        <v>0.05515280701772647</v>
       </c>
       <c r="H14" t="n">
-        <v>0.03307085724047992</v>
+        <v>0.02901894782023856</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.0246404985988846</v>
+        <v>0.2806493460516831</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.05268009763488148</v>
+        <v>-0.008924192964144765</v>
       </c>
       <c r="K14" t="n">
-        <v>0.01960986702368907</v>
+        <v>0.01590378690918018</v>
       </c>
       <c r="L14" t="n">
-        <v>0.1265143597509155</v>
+        <v>-0.03043192147242368</v>
       </c>
       <c r="M14" t="n">
-        <v>0.03535199604169725</v>
+        <v>0.2465594051809464</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
-        <v>-0.03422786351058907</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>gdp_pop_urban_merged</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.4392329713618456</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.1940996913778291</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.0604906980583572</v>
-      </c>
-      <c r="E15" t="n">
-        <v>-0.03071466180415534</v>
-      </c>
-      <c r="F15" t="n">
-        <v>-0.04134193923629658</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1959009620477364</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.05515280701772651</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0.02901894782023856</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0.2806493460516831</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-0.008924192964144761</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.01590378690918017</v>
-      </c>
-      <c r="M15" t="n">
-        <v>-0.03043192147242368</v>
-      </c>
-      <c r="N15" t="n">
-        <v>-0.03422786351058907</v>
-      </c>
-      <c r="O15" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>